<commit_message>
update file excel upload user
</commit_message>
<xml_diff>
--- a/data/bulk-upload-users/upload-users-invalid-data.xlsx
+++ b/data/bulk-upload-users/upload-users-invalid-data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cabe-1078\Desktop\Noted_CAB_2026\Data_Test_WUPoint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F5C142A-7035-41F3-B1D2-E2ECC8066882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2EDADF7-5293-4358-AAED-A1C92945F2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>no</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>firstName</t>
   </si>
@@ -41,6 +38,15 @@
   </si>
   <si>
     <t>phoneNumber</t>
+  </si>
+  <si>
+    <t>remark:</t>
+  </si>
+  <si>
+    <t>PASSPORT</t>
+  </si>
+  <si>
+    <t>NID</t>
   </si>
 </sst>
 </file>
@@ -69,27 +75,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -98,7 +89,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -403,30 +394,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F5" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>